<commit_message>
Cierre Fase 3: resultados regenerados (063 y 466 con ROI nueva) y documentacion actualizada
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_268_EXP3_FAPS2_40V/contracciones.xlsx
+++ b/data/processed_data/Video_268_EXP3_FAPS2_40V/contracciones.xlsx
@@ -1,18 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="estab_Video_268_EXP3_FAPS2" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resumen_Video_268_EXP3_FAP" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ritmo_Video_268_EXP3_FAPS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grilla_Video_268_EXP3_FAP" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eventos_Video_268_EXP3_FAP" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cinetica_Video_268_EXP3_FAP" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="estab_Video_268_EXP3_FAPS2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="resumen_Video_268_EXP3_FAP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ritmo_Video_268_EXP3_FAPS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="trenes_Video_268_EXP3_FAP" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="grilla_Video_268_EXP3_FAP" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="eventos_Video_268_EXP3_FAP" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="cinetica_Video_268_EXP3_FAP" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="cin_grupos_Video_268_EXP3_F" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,13 +24,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +44,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +52,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,22 +436,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>k</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>umbral_px</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>eventos</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>falsos_control</t>
         </is>
@@ -776,288 +790,323 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD2"/>
+  <dimension ref="A1:BK2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>canal</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>fps</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>n_frames</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>duracion_s</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>signo</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ruido_canal_px</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ruido_grosor_px</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>n_eventos</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>k_usado</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>k_automatico</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>hay_meseta</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>meseta_motivo</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>meseta_k_rango</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>conteo_reportable</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>intervalo_mediano_s</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>amplitud_traslacion_px</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>ritmo</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>fps_medido</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>adelgazamiento_px</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>adelgazamiento_sigma</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>retardo_adelgazamiento_s</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>cociente_adelg_trasl_pct</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>adelgazamiento_robusto_px</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>adelgazamiento_robusto_sigma</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>cociente_robusto_pct</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>blur_px</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>blur_sigma</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>cinetica_grupo_principal</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>cinetica_min_frames</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>n_eventos_cinetica</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>amplitud_relativa_pct</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>amplitud_relativa_iqr_pct</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_n_medibles</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_n_medibles</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida_pct</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>fotogramas_low_quality</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>eventos_junto_a_hueco</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>win_s_usado</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>win_s_automatico</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>duracion_evento_max_s</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>ventana_corta</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>conteo_por_ventana</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>conteo_estable_ventana</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>mesetas</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>ruido_borde_sup_px</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>ruido_borde_inf_px</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>cociente_ruido_bordes</t>
         </is>
       </c>
     </row>
@@ -1118,17 +1167,24 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{'n_eventos': 6, 'hay_estimulacion': True, 'estimulados': array([0, 1, 2, 3, 4, 5]), 'espontaneos': array([], dtype=int64), 'jitter_limitado_por_resolucion': True, 'z': 19.287, 'p_valor': 0.004975124378109453, 'periodo_grilla_s': 10.0108, 'periodo_s': 9.9999, 'periodo_err_s': 0.0023, 'frecuencia_Hz': 0.1, 'frecuencia_err_Hz': 2.3e-05, 'jitter_s': np.float64(0.00962), 'tolerancia_s': 0.0667, 'n_estimulados': 6, 'n_ranuras': 6, 'tasa_captura_pct': 100.0, 'tren_inicio_s': 12.667, 'tren_fin_s': 62.665, 'estimulados_dudosos': array([], dtype=int64), 'resumen_grupos':          grupo  n  ...  amplitud_mediana_px  amplitud_IQR_px
-0  estimulados  6  ...               1.5469             0.09
+          <t>{'n_eventos': 6, 'fuente_tiempo': 'inicio (onset 10 %) en 6 de 6 eventos; pico en el resto', 'modo_busqueda': 'dirigida', 'trenes':    tren           busqueda  ... inicio_s   fin_s
+0     1  dirigida a 0.1 Hz  ...   12.606  62.611
+[1 rows x 17 columns], 'dudosos': Empty DataFrame
+Columns: []
+Index: [], 'sacados_tiempo_amplitud': Empty DataFrame
+Columns: []
+Index: [], 'grupo_por_evento': array(['estimulados', 'estimulados', 'estimulados', 'estimulados',
+       'estimulados', 'estimulados'], dtype=object), 'tren_por_evento': array([1, 1, 1, 1, 1, 1]), 'estimulados': array([0, 1, 2, 3, 4, 5]), 'estimulados_dudosos': array([], dtype=int64), 'espontaneos': array([], dtype=int64), 'hay_estimulacion': True, 'n_trenes_estimulados': 1, 'tren_principal': 1, 'veredicto': 'enganchado a la frecuencia configurada (0.1 Hz)', 'z': 19.289, 'p_valor': 0.000999000999000999, 'periodo_grilla_s': 9.9782, 'periodo_s': 10.00132, 'periodo_err_s': 0.0023, 'frecuencia_Hz': 0.09999, 'frecuencia_err_Hz': 2.3e-05, 'jitter_s': np.float64(0.00962), 'tolerancia_s': 0.0667, 'n_estimulados': 6, 'n_ranuras': 6, 'tasa_captura_pct': 100.0, 'tren_inicio_s': 12.606, 'tren_fin_s': 62.611, 'jitter_limitado_por_resolucion': True, 'resumen_grupos':          grupo  n  t_inicio_s  ...  CV_intervalo_pct  amplitud_mediana_px  amplitud_IQR_px
+0  estimulados  6       12.61  ...               0.1               1.5469             0.09
 [1 rows x 10 columns], 'espontaneas_instantanea': Empty DataFrame
 Columns: [tiempo_s, intervalo_s, frecuencia_Hz]
-Index: [], 'grilla':    ranura  t_esperado_s  t_medido_s  error_s  capturada
-0       1       12.6658     12.6667  0.00087       True
-1       2       22.6657     22.6650 -0.00070       True
-2       3       32.6656     32.6650 -0.00060       True
-3       4       42.6655     42.6650 -0.00051       True
-4       5       52.6654     52.6667  0.00125       True
-5       6       62.6653     62.6650 -0.00032       True}</t>
+Index: [], 'grilla':    tren  ranura  t_esperado_s  t_medido_s  error_s  capturada
+0     1       1       12.6098     12.6059 -0.00392       True
+1     1       2       22.6111     22.6109 -0.00022       True
+2     1       3       32.6124     32.6196  0.00714       True
+3     1       4       42.6138     42.6104 -0.00335       True
+4     1       5       52.6151     52.6208  0.00575       True
+5     1       6       62.6164     62.6110 -0.00540       True}</t>
         </is>
       </c>
       <c r="R2" t="n">
@@ -1161,92 +1217,115 @@
       <c r="AA2" t="n">
         <v>15.70360888323099</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="AC2" t="n">
         <v>5</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE2" t="n">
         <v>0.5749451235599785</v>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>0.5636-0.5973</t>
         </is>
       </c>
-      <c r="AE2" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF2" t="n">
+      <c r="AG2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
         <v>2</v>
       </c>
-      <c r="AG2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="n">
+      <c r="AJ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="n">
         <v>0.1008333333333304</v>
       </c>
-      <c r="AL2" t="n">
-        <v>6</v>
-      </c>
-      <c r="AM2" t="n">
+      <c r="AO2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
         <v>2</v>
       </c>
-      <c r="AN2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR2" t="n">
+      <c r="AR2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="n">
         <v>0.1000000000000014</v>
       </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>TTP: 2 fotogramas (&lt; 5); solo cota TTP &lt; 101 ms; RT50: 2 fotogramas (&lt; 5); solo cota RT50 &lt; 100 ms</t>
-        </is>
-      </c>
-      <c r="AT2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW2" t="n">
-        <v>0</v>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>TTP: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 101 ms; RT50: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 100 ms</t>
+        </is>
       </c>
       <c r="AX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="n">
         <v>2</v>
       </c>
-      <c r="AY2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AZ2" t="n">
+      <c r="BC2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BD2" t="n">
         <v>0.5999999999999659</v>
       </c>
-      <c r="BA2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BB2" t="inlineStr">
+      <c r="BE2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="inlineStr">
         <is>
           <t>1.5 s: 6 | 2 s: 6 | 3 s: 6</t>
         </is>
       </c>
-      <c r="BC2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BD2" t="inlineStr">
+      <c r="BG2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH2" t="inlineStr">
         <is>
           <t>6 ev en k=5.846-24.421</t>
         </is>
+      </c>
+      <c r="BI2" t="n">
+        <v>0.07635389999996427</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>0.04017845999985895</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>1.900369003695819</v>
       </c>
     </row>
   </sheetData>
@@ -1264,52 +1343,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>t_inicio_s</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>t_fin_s</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>intervalo_mediano_s</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>intervalo_IQR_s</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>frecuencia_mediana_Hz</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>CV_intervalo_pct</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>amplitud_mediana_px</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>amplitud_IQR_px</t>
         </is>
@@ -1325,22 +1404,22 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>12.67</v>
+        <v>12.61</v>
       </c>
       <c r="D2" t="n">
-        <v>62.67</v>
+        <v>62.61</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>10.005</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0017</v>
+        <v>0.0179</v>
       </c>
       <c r="G2" t="n">
+        <v>0.0999</v>
+      </c>
+      <c r="H2" t="n">
         <v>0.1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>1.5469</v>
@@ -1360,33 +1439,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ranura</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>t_esperado_s</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>t_medido_s</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>error_s</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>capturada</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>tren</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>busqueda</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>veredicto</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>clasificacion</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>periodo_s</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>periodo_err_s</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>frecuencia_Hz</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>jitter_ms</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>z</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>p_valor</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>n_eventos_tren</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>n_ranuras</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>captura_pct</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>n_dudosos</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>n_sacados_tiempo_amplitud</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>inicio_s</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>fin_s</t>
         </is>
       </c>
     </row>
@@ -1394,102 +1533,59 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
-        <v>12.6658</v>
-      </c>
-      <c r="C2" t="n">
-        <v>12.6667</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.00087</v>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>22.6657</v>
-      </c>
-      <c r="C3" t="n">
-        <v>22.665</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-0.0007</v>
-      </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>32.6656</v>
-      </c>
-      <c r="C4" t="n">
-        <v>32.665</v>
-      </c>
-      <c r="D4" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
-      <c r="E4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="n">
-        <v>42.6655</v>
-      </c>
-      <c r="C5" t="n">
-        <v>42.665</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-0.00051</v>
-      </c>
-      <c r="E5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="n">
-        <v>52.6654</v>
-      </c>
-      <c r="C6" t="n">
-        <v>52.6667</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.00125</v>
-      </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="n">
-        <v>62.6653</v>
-      </c>
-      <c r="C7" t="n">
-        <v>62.665</v>
-      </c>
-      <c r="D7" t="n">
-        <v>-0.00032</v>
-      </c>
-      <c r="E7" t="b">
-        <v>1</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dirigida a 0.1 Hz</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>enganchado a la frecuencia configurada (0.1 Hz)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>10.00132</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.09999</v>
+      </c>
+      <c r="H2" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="I2" t="n">
+        <v>19.289</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.000999000999000999</v>
+      </c>
+      <c r="K2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2" t="n">
+        <v>6</v>
+      </c>
+      <c r="M2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>12.606</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>62.611</v>
       </c>
     </row>
   </sheetData>
@@ -1503,28 +1599,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>evento</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>tiempo_s</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>amplitud_px</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>junto_a_hueco</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>tren</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ranura</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>t_esperado_s</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>t_medido_s</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>error_s</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>capturada</t>
         </is>
       </c>
     </row>
@@ -1533,83 +1639,119 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>12.66666666666667</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1.442799999999977</v>
-      </c>
-      <c r="D2" t="b">
-        <v>0</v>
+        <v>12.6098</v>
+      </c>
+      <c r="D2" t="n">
+        <v>12.6059</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.00392</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
-        <v>22.665</v>
-      </c>
       <c r="C3" t="n">
-        <v>1.623500000000035</v>
-      </c>
-      <c r="D3" t="b">
-        <v>0</v>
+        <v>22.6111</v>
+      </c>
+      <c r="D3" t="n">
+        <v>22.6109</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-0.00022</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
-        <v>32.665</v>
-      </c>
       <c r="C4" t="n">
-        <v>1.563000000000045</v>
-      </c>
-      <c r="D4" t="b">
-        <v>0</v>
+        <v>32.6124</v>
+      </c>
+      <c r="D4" t="n">
+        <v>32.6196</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.00714</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
-        <v>42.66500000000001</v>
-      </c>
       <c r="C5" t="n">
-        <v>1.621499999999969</v>
-      </c>
-      <c r="D5" t="b">
-        <v>0</v>
+        <v>42.6138</v>
+      </c>
+      <c r="D5" t="n">
+        <v>42.6104</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.00335</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
-        <v>52.66666666666667</v>
-      </c>
       <c r="C6" t="n">
-        <v>1.530699999999968</v>
-      </c>
-      <c r="D6" t="b">
-        <v>0</v>
+        <v>52.6151</v>
+      </c>
+      <c r="D6" t="n">
+        <v>52.6208</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.00575</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B7" t="n">
-        <v>62.66500000000001</v>
+        <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>1.512299999999982</v>
-      </c>
-      <c r="D7" t="b">
-        <v>0</v>
+        <v>62.6164</v>
+      </c>
+      <c r="D7" t="n">
+        <v>62.611</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.0054</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1623,118 +1765,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>evento</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>grupo</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>frame_pico</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tiempo_s</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>amplitud_px</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>grosor_reposo_px</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>amplitud_relativa_pct</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>meseta_pico_frames</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>onset_s</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>ttp_frames</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>ttp_s</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>ttp_min_s</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>ttp_max_s</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>ttp_medible</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>rt50_frames</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>rt50_s</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>rt50_min_s</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>rt50_max_s</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>rt50_medible</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>offset_s</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>duracion_frames</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>duracion_s</t>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>junto_a_hueco</t>
         </is>
       </c>
     </row>
@@ -1742,420 +1794,911 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>estimulados</t>
-        </is>
+      <c r="B2" t="n">
+        <v>12.66666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>360</v>
-      </c>
-      <c r="D2" t="n">
-        <v>12.66666666666667</v>
-      </c>
-      <c r="E2" t="n">
         <v>1.442799999999977</v>
       </c>
-      <c r="F2" t="n">
-        <v>268.9955357766779</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.5363657786491298</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>12.60587210537497</v>
-      </c>
-      <c r="J2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.06079456129169714</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.09999999999999964</v>
-      </c>
-      <c r="N2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>2</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.06528735632183391</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.1000000000000014</v>
-      </c>
-      <c r="S2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>12.84246013667425</v>
-      </c>
-      <c r="U2" t="n">
-        <v>8</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.2365880312992772</v>
+      <c r="D2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>estimulados</t>
-        </is>
+      <c r="B3" t="n">
+        <v>22.665</v>
       </c>
       <c r="C3" t="n">
-        <v>660</v>
-      </c>
-      <c r="D3" t="n">
-        <v>22.665</v>
-      </c>
-      <c r="E3" t="n">
         <v>1.623500000000035</v>
       </c>
-      <c r="F3" t="n">
-        <v>269.0874972083027</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.6033353525687117</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>22.61089061256961</v>
-      </c>
-      <c r="J3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.05410938743038685</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.09999999999999787</v>
-      </c>
-      <c r="N3" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>3</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.0675953466851773</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.03166666666666984</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.1333333333333293</v>
-      </c>
-      <c r="S3" t="b">
-        <v>0</v>
-      </c>
-      <c r="T3" t="n">
-        <v>22.89679924242426</v>
-      </c>
-      <c r="U3" t="n">
-        <v>9</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.2859086298546458</v>
+      <c r="D3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>estimulados</t>
-        </is>
+      <c r="B4" t="n">
+        <v>32.665</v>
       </c>
       <c r="C4" t="n">
-        <v>960</v>
-      </c>
-      <c r="D4" t="n">
-        <v>32.665</v>
-      </c>
-      <c r="E4" t="n">
         <v>1.563000000000045</v>
       </c>
-      <c r="F4" t="n">
-        <v>269.0172640818902</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.5810036041122848</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>32.61957319163524</v>
-      </c>
-      <c r="J4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.0454268083647591</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.1000000000000014</v>
-      </c>
-      <c r="N4" t="b">
-        <v>0</v>
-      </c>
-      <c r="O4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.06199330380681545</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.1000000000000014</v>
-      </c>
-      <c r="S4" t="b">
-        <v>0</v>
-      </c>
-      <c r="T4" t="n">
-        <v>32.76201586214767</v>
-      </c>
-      <c r="U4" t="n">
-        <v>5</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.1424426705124304</v>
+      <c r="D4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>estimulados</t>
-        </is>
+      <c r="B5" t="n">
+        <v>42.66500000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>1260</v>
-      </c>
-      <c r="D5" t="n">
-        <v>42.66500000000001</v>
-      </c>
-      <c r="E5" t="n">
         <v>1.621499999999969</v>
       </c>
-      <c r="F5" t="n">
-        <v>269.0239091961759</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.6027345319770627</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" t="n">
-        <v>42.61040143705093</v>
-      </c>
-      <c r="J5" t="n">
-        <v>2</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.0545985629490815</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.1016666666666595</v>
-      </c>
-      <c r="N5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>2</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.06325072132396059</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0.1000000000000014</v>
-      </c>
-      <c r="S5" t="b">
-        <v>0</v>
-      </c>
-      <c r="T5" t="n">
-        <v>43.01668168168166</v>
-      </c>
-      <c r="U5" t="n">
-        <v>13</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0.4062802446307288</v>
+      <c r="D5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>estimulados</t>
-        </is>
+      <c r="B6" t="n">
+        <v>52.66666666666667</v>
       </c>
       <c r="C6" t="n">
-        <v>1560</v>
-      </c>
-      <c r="D6" t="n">
-        <v>52.66666666666667</v>
-      </c>
-      <c r="E6" t="n">
         <v>1.530699999999968</v>
       </c>
-      <c r="F6" t="n">
-        <v>269.0694216175021</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.5688866430076722</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>52.6208276154172</v>
-      </c>
-      <c r="J6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.04583905124947307</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.1016666666666666</v>
-      </c>
-      <c r="N6" t="b">
-        <v>0</v>
-      </c>
-      <c r="O6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.06302771530314999</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.09999999999998721</v>
-      </c>
-      <c r="S6" t="b">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
-        <v>53.01905769230767</v>
-      </c>
-      <c r="U6" t="n">
-        <v>13</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0.3982300768904707</v>
+      <c r="D6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
         <v>6</v>
       </c>
+      <c r="B7" t="n">
+        <v>62.66500000000001</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.512299999999982</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>evento</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>grupo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tren</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>frame_pico</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tiempo_s</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>grosor_reposo_px</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>amplitud_relativa_pct</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>meseta_pico_frames</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>onset_s</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_frames</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_s</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_min_s</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_max_s</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_medible</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_frames</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_s</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_min_s</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_max_s</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_medible</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>offset_s</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>duracion_frames</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>duracion_s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>360</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12.66666666666667</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.442799999999977</v>
+      </c>
+      <c r="G2" t="n">
+        <v>268.9955357766779</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.5363657786491298</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>12.60587210537497</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.06079456129169714</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.09999999999999964</v>
+      </c>
+      <c r="O2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.06528735632183391</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="T2" t="b">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>12.84246013667425</v>
+      </c>
+      <c r="V2" t="n">
+        <v>8</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.2365880312992772</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>660</v>
+      </c>
+      <c r="E3" t="n">
+        <v>22.665</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.623500000000035</v>
+      </c>
+      <c r="G3" t="n">
+        <v>269.0874972083027</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.6033353525687117</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>22.61089061256961</v>
+      </c>
+      <c r="K3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.05410938743038685</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.09999999999999787</v>
+      </c>
+      <c r="O3" t="b">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.0675953466851773</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.03166666666666984</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.1333333333333293</v>
+      </c>
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>22.89679924242426</v>
+      </c>
+      <c r="V3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.2859086298546458</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>960</v>
+      </c>
+      <c r="E4" t="n">
+        <v>32.665</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.563000000000045</v>
+      </c>
+      <c r="G4" t="n">
+        <v>269.0172640818901</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.5810036041122849</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>32.61957319163524</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0454268083647591</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="O4" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.06199330380681545</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="T4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>32.76201586214767</v>
+      </c>
+      <c r="V4" t="n">
+        <v>5</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.1424426705124304</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E5" t="n">
+        <v>42.66500000000001</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.621499999999969</v>
+      </c>
+      <c r="G5" t="n">
+        <v>269.0239091961759</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.6027345319770627</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>42.61040143705093</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0545985629490815</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.1016666666666595</v>
+      </c>
+      <c r="O5" t="b">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.06325072132396059</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>43.01668168168166</v>
+      </c>
+      <c r="V5" t="n">
+        <v>13</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.4062802446307288</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1560</v>
+      </c>
+      <c r="E6" t="n">
+        <v>52.66666666666667</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.530699999999968</v>
+      </c>
+      <c r="G6" t="n">
+        <v>269.0694216175021</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.5688866430076722</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>52.6208276154172</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.04583905124947307</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.1016666666666666</v>
+      </c>
+      <c r="O6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.06302771530314999</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.09999999999998721</v>
+      </c>
+      <c r="T6" t="b">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>53.01905769230767</v>
+      </c>
+      <c r="V6" t="n">
+        <v>13</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.3982300768904707</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>estimulados</t>
         </is>
       </c>
       <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
         <v>1850</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>62.66500000000001</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>1.512299999999982</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>269.1492529969205</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>0.5618815520239564</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>2</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>62.610998552822</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>2</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>0.0540014471780097</v>
       </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
       <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
         <v>0.1333333333333258</v>
       </c>
-      <c r="N7" t="b">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
+      <c r="O7" t="b">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
         <v>2</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>0.06252761266387097</v>
       </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
       <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
         <v>0.1000000000000014</v>
       </c>
-      <c r="S7" t="b">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
+      <c r="T7" t="b">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
         <v>63.06194039145907</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>14</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>0.4509418386370712</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>grupo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>cinetica_min_frames</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>n_eventos_cinetica</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>amplitud_relativa_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>amplitud_relativa_iqr_pct</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_n_eventos</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_n_medibles</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_frames_mediana</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_reportable</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_s</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_iqr_s</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_cota_inf_s</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ttp_cota_sup_s</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_n_eventos</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_n_medibles</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_frames_mediana</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_reportable</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_s</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_iqr_s</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_cota_inf_s</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>rt50_cota_sup_s</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>cinetica_motivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>todos</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.5749451235599785</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.5636-0.5973</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.1008333333333304</v>
+      </c>
+      <c r="N2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>TTP: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 101 ms; RT50: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 100 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.5749451235599785</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.5636-0.5973</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.1008333333333304</v>
+      </c>
+      <c r="N3" t="n">
+        <v>6</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q3" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>TTP: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 101 ms; RT50: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 100 ms</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>